<commit_message>
Update execution counts and outputs in Research Analysis notebook; replace error messages with results
Signed-off-by: Merite-M <mucyomerite@gmail.com>
</commit_message>
<xml_diff>
--- a/Student Perceptions of AI vs. Human Grading (Responses) (1).xlsx
+++ b/Student Perceptions of AI vs. Human Grading (Responses) (1).xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HP\Desktop\Kepler Courses\Statistics and Probability for Business\Statistics_Research_Project\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2A658D11-6F05-4593-A824-CC85D4E47120}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B1C3F322-F5B1-4232-80D0-45AB116B7A32}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="538" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="555" uniqueCount="47">
   <si>
     <t>Timestamp</t>
   </si>
@@ -739,8 +739,8 @@
       <c r="H7" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="I7" s="3" t="s">
-        <v>10</v>
+      <c r="I7" s="4" t="s">
+        <v>27</v>
       </c>
       <c r="J7" s="3" t="s">
         <v>11</v>
@@ -833,7 +833,9 @@
       <c r="H10" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="I10" s="4"/>
+      <c r="I10" s="4" t="s">
+        <v>35</v>
+      </c>
       <c r="J10" s="3" t="s">
         <v>11</v>
       </c>
@@ -927,7 +929,9 @@
       <c r="H13" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="I13" s="4"/>
+      <c r="I13" s="4" t="s">
+        <v>35</v>
+      </c>
       <c r="J13" s="3" t="s">
         <v>11</v>
       </c>
@@ -1181,8 +1185,8 @@
       <c r="H21" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="I21" s="3" t="s">
-        <v>27</v>
+      <c r="I21" s="4" t="s">
+        <v>35</v>
       </c>
       <c r="J21" s="3" t="s">
         <v>11</v>
@@ -1373,8 +1377,8 @@
       <c r="H27" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="I27" s="3" t="s">
-        <v>27</v>
+      <c r="I27" s="4" t="s">
+        <v>35</v>
       </c>
       <c r="J27" s="3" t="s">
         <v>11</v>
@@ -1533,8 +1537,8 @@
       <c r="H32" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="I32" s="3" t="s">
-        <v>27</v>
+      <c r="I32" s="4" t="s">
+        <v>35</v>
       </c>
       <c r="J32" s="3" t="s">
         <v>11</v>
@@ -1629,7 +1633,9 @@
       <c r="H35" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="I35" s="4"/>
+      <c r="I35" s="4" t="s">
+        <v>35</v>
+      </c>
       <c r="J35" s="3" t="s">
         <v>11</v>
       </c>
@@ -1723,8 +1729,8 @@
       <c r="H38" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="I38" s="3" t="s">
-        <v>10</v>
+      <c r="I38" s="4" t="s">
+        <v>35</v>
       </c>
       <c r="J38" s="3" t="s">
         <v>11</v>
@@ -1755,7 +1761,9 @@
       <c r="H39" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="I39" s="4"/>
+      <c r="I39" s="4" t="s">
+        <v>35</v>
+      </c>
       <c r="J39" s="3" t="s">
         <v>11</v>
       </c>
@@ -1881,7 +1889,9 @@
       <c r="H43" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="I43" s="4"/>
+      <c r="I43" s="4" t="s">
+        <v>35</v>
+      </c>
       <c r="J43" s="3" t="s">
         <v>11</v>
       </c>
@@ -1975,7 +1985,9 @@
       <c r="H46" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="I46" s="4"/>
+      <c r="I46" s="4" t="s">
+        <v>35</v>
+      </c>
       <c r="J46" s="3" t="s">
         <v>11</v>
       </c>
@@ -2069,7 +2081,9 @@
       <c r="H49" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="I49" s="3"/>
+      <c r="I49" s="4" t="s">
+        <v>35</v>
+      </c>
       <c r="J49" s="3" t="s">
         <v>11</v>
       </c>
@@ -2099,7 +2113,9 @@
       <c r="H50" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="I50" s="3"/>
+      <c r="I50" s="4" t="s">
+        <v>35</v>
+      </c>
       <c r="J50" s="3" t="s">
         <v>11</v>
       </c>
@@ -2417,7 +2433,9 @@
       <c r="H60" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="I60" s="3"/>
+      <c r="I60" s="4" t="s">
+        <v>35</v>
+      </c>
       <c r="J60" s="3" t="s">
         <v>11</v>
       </c>
@@ -2671,7 +2689,9 @@
       <c r="H68" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="I68" s="4"/>
+      <c r="I68" s="4" t="s">
+        <v>35</v>
+      </c>
       <c r="J68" s="3" t="s">
         <v>11</v>
       </c>
@@ -2701,7 +2721,9 @@
       <c r="H69" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="I69" s="4"/>
+      <c r="I69" s="4" t="s">
+        <v>35</v>
+      </c>
       <c r="J69" s="3" t="s">
         <v>11</v>
       </c>
@@ -2763,7 +2785,9 @@
       <c r="H71" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="I71" s="3"/>
+      <c r="I71" s="4" t="s">
+        <v>35</v>
+      </c>
       <c r="J71" s="3" t="s">
         <v>11</v>
       </c>
@@ -2857,7 +2881,9 @@
       <c r="H74" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="I74" s="4"/>
+      <c r="I74" s="4" t="s">
+        <v>35</v>
+      </c>
       <c r="J74" s="3" t="s">
         <v>11</v>
       </c>
@@ -2951,7 +2977,9 @@
       <c r="H77" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="I77" s="4"/>
+      <c r="I77" s="4" t="s">
+        <v>35</v>
+      </c>
       <c r="J77" s="3" t="s">
         <v>11</v>
       </c>
@@ -2981,7 +3009,9 @@
       <c r="H78" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="I78" s="4"/>
+      <c r="I78" s="4" t="s">
+        <v>35</v>
+      </c>
       <c r="J78" s="3" t="s">
         <v>11</v>
       </c>
@@ -3043,7 +3073,9 @@
       <c r="H80" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="I80" s="4"/>
+      <c r="I80" s="4" t="s">
+        <v>35</v>
+      </c>
       <c r="J80" s="3" t="s">
         <v>11</v>
       </c>
@@ -3073,7 +3105,9 @@
       <c r="H81" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="I81" s="4"/>
+      <c r="I81" s="4" t="s">
+        <v>35</v>
+      </c>
       <c r="J81" s="3" t="s">
         <v>11</v>
       </c>
@@ -3327,8 +3361,8 @@
       <c r="H89" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="I89" s="3" t="s">
-        <v>27</v>
+      <c r="I89" s="4" t="s">
+        <v>35</v>
       </c>
       <c r="J89" s="3" t="s">
         <v>11</v>

</xml_diff>